<commit_message>
chore: update outputs for all modules (M1→M7)
- pipeline/outputs/: module1-7 structured outputs + pipeline_result.json
- module7/output/: updated business.pdf and business.xlsx
- removed module4/.env.example

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Desktop/bootcamp ai/module7/output/business.xlsx
+++ b/Desktop/bootcamp ai/module7/output/business.xlsx
@@ -496,13 +496,13 @@
         </is>
       </c>
       <c r="B2" s="3" t="n">
-        <v>154208</v>
+        <v>149582</v>
       </c>
       <c r="C2" s="3" t="n">
-        <v>169628.8</v>
+        <v>164540.2</v>
       </c>
       <c r="D2" s="3" t="n">
-        <v>186591.68</v>
+        <v>180994.22</v>
       </c>
     </row>
     <row r="3">
@@ -512,13 +512,13 @@
         </is>
       </c>
       <c r="B3" s="5" t="n">
-        <v>-1356661.443978205</v>
+        <v>-1315972.471160076</v>
       </c>
       <c r="C3" s="5" t="n">
-        <v>-1341240.643978205</v>
+        <v>-1301014.271160076</v>
       </c>
       <c r="D3" s="5" t="n">
-        <v>-1324277.763978205</v>
+        <v>-1284560.251160076</v>
       </c>
     </row>
     <row r="4">
@@ -528,13 +528,13 @@
         </is>
       </c>
       <c r="B4" s="6" t="n">
-        <v>-0.8979342651910667</v>
+        <v>-0.8979348752001032</v>
       </c>
       <c r="C4" s="6" t="n">
-        <v>-0.8877276917101733</v>
+        <v>-0.8877283627201135</v>
       </c>
       <c r="D4" s="6" t="n">
-        <v>-0.8765004608811907</v>
+        <v>-0.8765011989921248</v>
       </c>
     </row>
     <row r="5">
@@ -544,7 +544,7 @@
         </is>
       </c>
       <c r="B5" s="8" t="n">
-        <v>-3336741.412147151</v>
+        <v>-3236666.145409354</v>
       </c>
       <c r="C5" s="9" t="n"/>
       <c r="D5" s="9" t="n"/>

</xml_diff>

<commit_message>
chore: remove old module2/3 files + update all pipeline outputs
Removed (replaced by new agent2/agent3):
- module2/agents/{dxf,geometry,ifc,rule,step,validation}_agent.py
- module2/models/valve_model.py, module2/services/geometry_engine.py
- module3/blender_runner.py, module3/main.py
- pipeline/outputs/valve.{dxf,ifc,step} (now generated per run_id)

Updated outputs:
- pipeline/outputs/module2-7 JSON/PDF results
- module7/output/business.pdf + business.xlsx

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Desktop/bootcamp ai/module7/output/business.xlsx
+++ b/Desktop/bootcamp ai/module7/output/business.xlsx
@@ -496,13 +496,13 @@
         </is>
       </c>
       <c r="B2" s="3" t="n">
-        <v>149582</v>
+        <v>151678</v>
       </c>
       <c r="C2" s="3" t="n">
-        <v>164540.2</v>
+        <v>166845.8</v>
       </c>
       <c r="D2" s="3" t="n">
-        <v>180994.22</v>
+        <v>183530.38</v>
       </c>
     </row>
     <row r="3">
@@ -512,13 +512,13 @@
         </is>
       </c>
       <c r="B3" s="5" t="n">
-        <v>-1315972.471160076</v>
+        <v>-1334404.444836006</v>
       </c>
       <c r="C3" s="5" t="n">
-        <v>-1301014.271160076</v>
+        <v>-1319236.644836006</v>
       </c>
       <c r="D3" s="5" t="n">
-        <v>-1284560.251160076</v>
+        <v>-1302552.064836006</v>
       </c>
     </row>
     <row r="4">
@@ -528,13 +528,13 @@
         </is>
       </c>
       <c r="B4" s="6" t="n">
-        <v>-0.8979348752001032</v>
+        <v>-0.8979343302741605</v>
       </c>
       <c r="C4" s="6" t="n">
-        <v>-0.8877283627201135</v>
+        <v>-0.8877277633015764</v>
       </c>
       <c r="D4" s="6" t="n">
-        <v>-0.8765011989921248</v>
+        <v>-0.876500539631734</v>
       </c>
     </row>
     <row r="5">
@@ -544,7 +544,7 @@
         </is>
       </c>
       <c r="B5" s="8" t="n">
-        <v>-3236666.145409354</v>
+        <v>-3281999.81397985</v>
       </c>
       <c r="C5" s="9" t="n"/>
       <c r="D5" s="9" t="n"/>

</xml_diff>